<commit_message>
Add review comment workflow
</commit_message>
<xml_diff>
--- a/LeaguePost/league_team_list.xlsx
+++ b/LeaguePost/league_team_list.xlsx
@@ -5,22 +5,22 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\python_apps\LeaguePost\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rmiop\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{175F6491-10C4-416F-9F8B-F43B9CBBD6F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE77D008-7415-420D-80A3-64CFDDEDAB7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4900" yWindow="760" windowWidth="14120" windowHeight="12620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22180" windowHeight="14140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="連盟チーム一覧" sheetId="1" r:id="rId1"/>
+    <sheet name="チーム一覧" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="57">
   <si>
     <t>チーム名</t>
   </si>
@@ -146,6 +146,66 @@
   </si>
   <si>
     <t>山口大</t>
+  </si>
+  <si>
+    <t>チームコード</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>toridai</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>torii</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>shimadai</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>kibikoku</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>okadai</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>okai</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>kawai</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>hirosyu</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>hirokoku</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>hirodai</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>hiroi</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>kaiho</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>shimoichi</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>yamadai</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
@@ -529,17 +589,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.25" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="5.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="12" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="14" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -558,8 +618,11 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="14" x14ac:dyDescent="0.2">
+      <c r="G1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -578,8 +641,11 @@
       <c r="F2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="14" x14ac:dyDescent="0.2">
+      <c r="G2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -598,8 +664,11 @@
       <c r="F3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="14" x14ac:dyDescent="0.2">
+      <c r="G3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -618,8 +687,11 @@
       <c r="F4" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="14" x14ac:dyDescent="0.2">
+      <c r="G4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -638,8 +710,11 @@
       <c r="F5" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="14" x14ac:dyDescent="0.2">
+      <c r="G5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="14" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -658,8 +733,11 @@
       <c r="F6" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="14" x14ac:dyDescent="0.2">
+      <c r="G6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="14" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -678,8 +756,11 @@
       <c r="F7" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="14" x14ac:dyDescent="0.2">
+      <c r="G7" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="14" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -698,8 +779,11 @@
       <c r="F8" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="14" x14ac:dyDescent="0.2">
+      <c r="G8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="14" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -718,8 +802,11 @@
       <c r="F9" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="14" x14ac:dyDescent="0.2">
+      <c r="G9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="14" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -738,8 +825,11 @@
       <c r="F10" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="14" x14ac:dyDescent="0.2">
+      <c r="G10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="14" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>31</v>
       </c>
@@ -758,8 +848,11 @@
       <c r="F11" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="14" x14ac:dyDescent="0.2">
+      <c r="G11" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="14" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>33</v>
       </c>
@@ -778,8 +871,11 @@
       <c r="F12" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="14" x14ac:dyDescent="0.2">
+      <c r="G12" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="14" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>35</v>
       </c>
@@ -798,8 +894,11 @@
       <c r="F13" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="14" x14ac:dyDescent="0.2">
+      <c r="G13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="14" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>37</v>
       </c>
@@ -818,8 +917,11 @@
       <c r="F14" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" ht="14" x14ac:dyDescent="0.2">
+      <c r="G14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="14" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>40</v>
       </c>
@@ -837,6 +939,9 @@
       </c>
       <c r="F15" t="s">
         <v>39</v>
+      </c>
+      <c r="G15" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>